<commit_message>
Populate presentation dataset: 40 verified voters and 16 realistic municipal proposals
</commit_message>
<xml_diff>
--- a/proposals.xlsx
+++ b/proposals.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Proposals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,25 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00E4C766"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B2A23"/>
-        <bgColor rgb="001B2A23"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -58,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,32 +413,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ward</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>desc</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>budget</t>
         </is>
@@ -467,36 +446,316 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Solar Lighting at Bus Stand</t>
+          <t>Anna Park Eco-Renovation &amp; Jogging Track</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Install 10 solar-powered lighting masts at bus stops.</t>
+          <t>Resurface 1.2km walking paths with porous eco-tiles, install solar LED pathway lights, and add shaded benches.</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>450000</v>
+        <v>1450000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Ward 1 — Anna Nagar</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Smart LED Streetlight Transition (Phase 2)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Replace 65 legacy sodium lamps with energy-efficient smart LED luminaires along residential 2nd &amp; 3rd Avenues.</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>880000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ward 1 — Anna Nagar</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Rainwater Harvesting &amp; Storm Drain Desilting</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Deep desilting of arterial stormwater conduits and installation of 8 percolation filtration chambers before monsoon.</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1120000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ward 1 — Anna Nagar</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Automated Solid Waste Compactor Station</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Deploy modern odor-free closed hydraulic refuse compactor on 6th Main Road for hygienic waste processing.</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1600000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Ward 2 — T Nagar</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Pedestrian Walkway Ramp</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Add accessible wheelchair ramps along market pedestrian zone.</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>350000</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pedestrian Plaza Expansion &amp; Pavement Upgrades</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Extend accessible bollard-protected tactile walkways, anti-skid paver tiles, and ornamental planters along Pondy Bazaar corridor.</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1850000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ward 2 — T Nagar</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Automated Two-Wheeler Parking Facility</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Construct a 40-slot automated stacked bike parking hub near Usman Road junction to eliminate sidewalk congestion.</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ward 2 — T Nagar</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Modern Public Sanitation &amp; Hygiene Complex</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Construct a 24x7 accessible public toilet with touchless sensor fittings and dedicated child/elderly care stalls.</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>750000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ward 2 — T Nagar</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Overhead Cable Trenching &amp; Underground Ducting</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Relocate haphazard overhead optical fiber cables into underground micro-ducts along Ranganathan Street cross-lanes.</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1380000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ward 3 — Adyar</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Adyar Riverfront Green Corridor &amp; Solar Lighting</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Install 45 standalone solar luminary poles and native avenue trees along the riverside pedestrian walkway.</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1250000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ward 3 — Adyar</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Aquifer Percolation Recharge Wells</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Construct 10 decentralized stormwater percolation recharge wells in low-lying residential sectors to prevent seasonal waterlogging.</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>920000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ward 3 — Adyar</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Elderly Wellness Park &amp; Outdoor Open-Air Gym</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Establish an outdoor rehabilitation gym with low-impact equipment, acupressure walking track, and first-aid kiosk.</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>680000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ward 3 — Adyar</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Community Aerobic Composting &amp; Biogas Unit</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Set up an aerobic community composting facility at Gandhi Nagar for local organic wet waste conversion.</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>840000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ward 4 — Mylapore</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Heritage Temple Tank Restoration &amp; Embankment Repair</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Restore historic stone embankments, install aeration water fountains, and desilt peripheral catchment feeders.</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1900000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Ward 4 — Mylapore</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Traffic Calming &amp; Heritage Lane Signage</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Install rubberized modular speed tables, retro-reflective heritage street signage, and bollards around temple squares.</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>550000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Ward 4 — Mylapore</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Secondary Drainage Pipeline &amp; Stormwater Interceptor</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Lay 800m high-density polyethylene pipeline to divert excess rainwater into temple tank reservoirs.</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1520000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ward 4 — Mylapore</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Solar-Powered E-Library &amp; Digital Study Centre</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Modernize the municipal reading room with 15 digital learning tablets, high-speed Wi-Fi, and 5kW rooftop solar panels.</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1050000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>